<commit_message>
auto(CY): 3h refresh 2026-05-16T08:42Z
</commit_message>
<xml_diff>
--- a/daily_report_2026-05-16.xlsx
+++ b/daily_report_2026-05-16.xlsx
@@ -642,8 +642,6 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
           <t>2026-05-16 05:20</t>
@@ -751,8 +749,6 @@
           <t>2026-03-08</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
           <t>2026-05-16 05:20</t>
@@ -860,8 +856,6 @@
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t>2026-05-16 05:20</t>
@@ -4478,8 +4472,6 @@
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
       <c r="M65" t="inlineStr">
         <is>
           <t>2026-05-16 05:20</t>
@@ -4595,8 +4587,6 @@
           <t>2026-05-10</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
       <c r="M67" t="inlineStr">
         <is>
           <t>2026-05-16 05:20</t>
@@ -5717,8 +5707,6 @@
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
       <c r="M85" t="inlineStr">
         <is>
           <t>2026-05-16 05:20</t>
@@ -5959,8 +5947,6 @@
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="inlineStr"/>
       <c r="M89" t="inlineStr">
         <is>
           <t>2026-05-16 05:20</t>
@@ -6251,7 +6237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M70"/>
+  <dimension ref="A1:M87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -9858,8 +9844,6 @@
           <t>2026-05-03</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
       <c r="M69" t="inlineStr">
         <is>
           <t>2026-05-16 06:17</t>
@@ -9918,6 +9902,910 @@
       <c r="M70" s="3" t="inlineStr">
         <is>
           <t>2026-05-16 06:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Μαυρικιος Αντρέας</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>ΟΙΚΟΛΟΓΟΙ</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Αντρέας Μαυρίκιος - Andreas Mavrikios</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>111609967364337</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>800373569774308</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>2026-05-16 08:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>Χαμπούλλας Ευγένιος</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>ΕΛΑΜ</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>157660994287097</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>4481282198796917</t>
+        </is>
+      </c>
+      <c r="G72" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="I72" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="J72" s="3" t="inlineStr"/>
+      <c r="K72" s="3" t="inlineStr"/>
+      <c r="L72" s="3" t="n"/>
+      <c r="M72" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 08:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Χαμπούλλας Ευγένιος</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>ΕΛΑΜ</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>157660994287097</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>4374884449433106</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>2026-05-16 08:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Χαμπούλλας Ευγένιος</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>ΕΛΑΜ</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>157660994287097</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>1283965546996339</t>
+        </is>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="I74" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="J74" s="3" t="inlineStr"/>
+      <c r="K74" s="3" t="inlineStr"/>
+      <c r="L74" s="3" t="n"/>
+      <c r="M74" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 08:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Αθανασιάδης Ζαχαρίας</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>ΕΛΑΜ</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Ζαχαρίας Αθανασιάδης</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>146231858570802</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>915311188208188</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>2026-05-16 08:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>574683626048556</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>2117437872160480</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="I76" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="J76" s="3" t="inlineStr"/>
+      <c r="K76" s="3" t="inlineStr"/>
+      <c r="L76" s="3" t="n"/>
+      <c r="M76" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 08:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>574683626048556</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>1594141958314551</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>2026-05-16 08:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>574683626048556</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>1536747531135576</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="I78" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="J78" s="3" t="inlineStr"/>
+      <c r="K78" s="3" t="inlineStr"/>
+      <c r="L78" s="3" t="n"/>
+      <c r="M78" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 08:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>754699914874253</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>1710761040097847</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>2026-05-16 08:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>574683626048556</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>1299287425628320</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="I80" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="J80" s="3" t="inlineStr"/>
+      <c r="K80" s="3" t="inlineStr"/>
+      <c r="L80" s="3" t="n"/>
+      <c r="M80" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 08:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>574683626048556</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>1514212826786750</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>2026-05-16 08:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>Βουτηρου Σάββας</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>ΣΗΚΟΥ ΠΑΝΩ</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Αμμόχωστος</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>Σαββας Βουτήρου - Savvas Voutirou</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>100936455330537</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>1299002585765427</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I82" s="3" t="n"/>
+      <c r="J82" s="3" t="inlineStr"/>
+      <c r="K82" s="3" t="inlineStr"/>
+      <c r="L82" s="3" t="n"/>
+      <c r="M82" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 07:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Άσπρης Άδαμος</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>ΔΗΚΟ</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Κερύνεια</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Adamos Aspris - Αδάμος Ασπρής</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>1544889622506869</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>1287137836934355</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>2026-05-16 07:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>Χατζηπαναγή Αρτέμης</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>ΕΝΕΡΓΟΙ ΠΟΛΙΤΕΣ</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>Αρτέμης Χατζηπαναγή</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>111255711940633</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>4323642054565212</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I84" s="3" t="n"/>
+      <c r="J84" s="3" t="inlineStr"/>
+      <c r="K84" s="3" t="inlineStr"/>
+      <c r="L84" s="3" t="n"/>
+      <c r="M84" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 07:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Παύλου Τίνα</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Τίνα Παύλου - Tina Pavlou</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>802383349636152</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>2718683645168629</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr"/>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>2026-05-16 07:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>Σαββίδης Χρύσανθος</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΚΟ</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>Χρύσανθος Σαββίδης</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>556192687867978</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>2071083287123146</t>
+        </is>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I86" s="3" t="n"/>
+      <c r="J86" s="3" t="inlineStr"/>
+      <c r="K86" s="3" t="inlineStr"/>
+      <c r="L86" s="3" t="n"/>
+      <c r="M86" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 07:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Αποστόλου Ανδρέας</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>ΔΗΚΟ</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Λάρνακα</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Ανδρέας Αποστόλου</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>502944236549149</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>1695784821453815</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr"/>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>2026-05-16 07:47</t>
         </is>
       </c>
     </row>
@@ -9992,6 +10880,23 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10003,13 +10908,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
@@ -10212,32 +11117,32 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Μηνά Πέτρος</t>
+          <t>Βουτηρου Σάββας</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>ΔΕΚ</t>
+          <t>ΣΗΚΟΥ ΠΑΝΩ</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Λεμεσός</t>
+          <t>Αμμόχωστος</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Athena astrologer</t>
+          <t>Σαββας Βουτήρου - Savvas Voutirou</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>1069759626211045</t>
+          <t>100936455330537</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>998326189395922</t>
+          <t>1299002585765427</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -10260,38 +11165,38 @@
         </is>
       </c>
       <c r="N4" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Μηνά Πέτρος</t>
+          <t>Γεωργιάδης Δήμος</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Λεμεσός</t>
+          <t>Κερύνεια</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Athena astrologer</t>
+          <t>Δήμος Γεωργιάδης</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1069759626211045</t>
+          <t>107513542170251</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1275910284745101</t>
+          <t>1286848666896373</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -10301,7 +11206,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -10312,38 +11217,38 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Μηνά Πέτρος</t>
+          <t>Γεωργιάδης Δήμος</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>ΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Λεμεσός</t>
+          <t>Κερύνεια</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Athena astrologer</t>
+          <t>Δήμος Γεωργιάδης</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>1069759626211045</t>
+          <t>107513542170251</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>1991042238452462</t>
+          <t>1303700075068172</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -10353,10 +11258,14 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="inlineStr"/>
       <c r="K6" s="3" t="inlineStr"/>
       <c r="L6" s="3" t="n"/>
@@ -10366,18 +11275,18 @@
         </is>
       </c>
       <c r="N6" s="3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Μηνά Πέτρος</t>
+          <t>Αθανασιάδης Ζαχαρίας</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ΔΕΚ</t>
+          <t>ΕΛΑΜ</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -10387,17 +11296,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Athena astrologer</t>
+          <t>Ζαχαρίας Αθανασιάδης</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1069759626211045</t>
+          <t>146231858570802</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2006149173307958</t>
+          <t>1330888802244834</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -10407,29 +11316,42 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>25,000–29,999</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Γεωργιάδης Δήμος</t>
+          <t>Άσπρης Άδαμος</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -10439,17 +11361,17 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Δήμος Γεωργιάδης</t>
+          <t>Adamos Aspris - Αδάμος Ασπρής</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>107513542170251</t>
+          <t>1544889622506869</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>1286848666896373</t>
+          <t>1287137836934355</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -10459,7 +11381,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="I8" s="3" t="n"/>
@@ -10472,38 +11394,38 @@
         </is>
       </c>
       <c r="N8" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Γεωργιάδης Δήμος</t>
+          <t>Χαμπούλλας Ευγένιος</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΕΛΑΜ</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Κερύνεια</t>
+          <t>Λεμεσός</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Δήμος Γεωργιάδης</t>
+          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>107513542170251</t>
+          <t>157660994287097</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1303700075068172</t>
+          <t>1032725159187111</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -10512,11 +11434,6 @@
         </is>
       </c>
       <c r="H9" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
         <is>
           <t>2026-05-15</t>
         </is>
@@ -10529,13 +11446,13 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Αθανασιάδης Ζαχαρίας</t>
+          <t>Χαμπούλλας Ευγένιος</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -10550,17 +11467,17 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Ζαχαρίας Αθανασιάδης</t>
+          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>146231858570802</t>
+          <t>157660994287097</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>1330888802244834</t>
+          <t>3440749736091343</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -10570,24 +11487,12 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>25,000–29,999</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>0–99</t>
-        </is>
-      </c>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr"/>
       <c r="L10" s="3" t="n"/>
       <c r="M10" s="3" t="inlineStr">
         <is>
@@ -10595,38 +11500,38 @@
         </is>
       </c>
       <c r="N10" s="3" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Χαμπούλλας Ευγένιος</t>
+          <t>Αποστόλου Ανδρέας</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ΕΛΑΜ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Λεμεσός</t>
+          <t>Λάρνακα</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
+          <t>Ανδρέας Αποστόλου</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>157660994287097</t>
+          <t>502944236549149</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1032725159187111</t>
+          <t>1695784821453815</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -10635,6 +11540,11 @@
         </is>
       </c>
       <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>2026-05-15</t>
         </is>
@@ -10647,38 +11557,38 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Χαμπούλλας Ευγένιος</t>
+          <t>Σαββίδης Χρύσανθος</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>ΕΛΑΜ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Λεμεσός</t>
+          <t>Πάφος</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
+          <t>Χρύσανθος Σαββίδης</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>157660994287097</t>
+          <t>556192687867978</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>3440749736091343</t>
+          <t>2071083287123146</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -10688,7 +11598,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="I12" s="3" t="n"/>
@@ -10701,38 +11611,38 @@
         </is>
       </c>
       <c r="N12" s="3" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Αποστόλου Ανδρέας</t>
+          <t>Φελλάς Μιχάλης</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Λάρνακα</t>
+          <t>Λεμεσός</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Ανδρέας Αποστόλου</t>
+          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>502944236549149</t>
+          <t>574683626048556</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2385960758575830</t>
+          <t>2460936817680213</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -10742,7 +11652,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -10753,13 +11668,13 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>21</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης</t>
+          <t>Ευαγγελου Αργυρός</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -10769,22 +11684,22 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Λεμεσός</t>
+          <t>Λάρνακα</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+          <t>Αργυρός Ευαγγέλου - Argyros Evangelou</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>574683626048556</t>
+          <t>595915680800838</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>2460936817680213</t>
+          <t>2039508410305874</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -10794,14 +11709,10 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="inlineStr"/>
       <c r="K14" s="3" t="inlineStr"/>
       <c r="L14" s="3" t="n"/>
@@ -10811,38 +11722,38 @@
         </is>
       </c>
       <c r="N14" s="3" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Ευαγγελου Αργυρός</t>
+          <t>Κορύτσα Μαρία</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΕΛΑΜ</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Λάρνακα</t>
+          <t>Αμμόχωστος</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Αργυρός Ευαγγέλου - Argyros Evangelou</t>
+          <t>Μαρία Κορυτσά</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>595915680800838</t>
+          <t>636019372933735</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2039508410305874</t>
+          <t>1296943101983207</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -10852,7 +11763,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -10863,7 +11774,7 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16">
@@ -10894,7 +11805,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>1296943101983207</t>
+          <t>813726091505369</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -10904,12 +11815,24 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="I16" s="3" t="n"/>
-      <c r="J16" s="3" t="inlineStr"/>
-      <c r="K16" s="3" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>1,000–1,999</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
       <c r="L16" s="3" t="n"/>
       <c r="M16" s="3" t="inlineStr">
         <is>
@@ -10923,32 +11846,32 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Κορύτσα Μαρία</t>
+          <t>Φελλάς Μιχάλης</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ΕΛΑΜ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Αμμόχωστος</t>
+          <t>Λεμεσός</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Μαρία Κορυτσά</t>
+          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>636019372933735</t>
+          <t>754699914874253</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>813726091505369</t>
+          <t>1271006601866511</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -10958,62 +11881,54 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>1,000–1,999</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>0–99</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
       <c r="N17" t="n">
-        <v>15</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Κωνσταντινου Κώστας</t>
+          <t>Φελλάς Μιχάλης</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>ΑΓΡΟΝΟΜΟΣ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Λευκωσία</t>
+          <t>Λεμεσός</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Special Inclusive Education - Ειδική και Ενιαία Εκπαίδευση</t>
+          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>699453867584289</t>
+          <t>754699914874253</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>876941465437111</t>
+          <t>2150144575829086</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -11026,7 +11941,11 @@
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="I18" s="3" t="n"/>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
       <c r="J18" s="3" t="inlineStr"/>
       <c r="K18" s="3" t="inlineStr"/>
       <c r="L18" s="3" t="n"/>
@@ -11036,13 +11955,13 @@
         </is>
       </c>
       <c r="N18" s="3" t="n">
-        <v>2</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης</t>
+          <t>Παύλου Τίνα</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -11052,22 +11971,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Λεμεσός</t>
+          <t>Λευκωσία</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+          <t>Τίνα Παύλου - Tina Pavlou</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>754699914874253</t>
+          <t>802383349636152</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1271006601866511</t>
+          <t>2718683645168629</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
@@ -11077,12 +11996,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -11093,13 +12007,13 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>79</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης</t>
+          <t>Παύλου Τίνα</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -11109,22 +12023,22 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Λεμεσός</t>
+          <t>Λευκωσία</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+          <t>Τίνα Παύλου - Tina Pavlou</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>754699914874253</t>
+          <t>802383349636152</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>2150144575829086</t>
+          <t>838326815506972</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -11151,18 +12065,18 @@
         </is>
       </c>
       <c r="N20" s="3" t="n">
-        <v>79</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ερωτοκρίτου Χριστιάνα</t>
+          <t>Παύλου Τίνα</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -11172,17 +12086,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Χριστιάνα Ερωτοκρίτου</t>
+          <t>Τίνα Παύλου - Tina Pavlou</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>771955332942116</t>
+          <t>802383349636152</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1625748798478075</t>
+          <t>1308821568004990</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -11192,7 +12106,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -11203,7 +12117,7 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22">
@@ -11234,7 +12148,7 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>838326815506972</t>
+          <t>939589268904899</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -11244,14 +12158,10 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="inlineStr"/>
       <c r="K22" s="3" t="inlineStr"/>
       <c r="L22" s="3" t="n"/>
@@ -11292,7 +12202,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1308821568004990</t>
+          <t>35380689674908199</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -11302,11 +12212,24 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>3,000–3,999</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
       <c r="M23" t="inlineStr">
         <is>
           <t>2026-05-14</t>
@@ -11319,32 +12242,32 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Παύλου Τίνα</t>
+          <t>Ελληνας Σάββας</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΑΜΔΗ</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Λευκωσία</t>
+          <t>Πάφος</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Τίνα Παύλου - Tina Pavlou</t>
+          <t>Έλληνας Σάββας</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>802383349636152</t>
+          <t>865790916625202</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>939589268904899</t>
+          <t>4446806865575192</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -11354,7 +12277,7 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="I24" s="3" t="n"/>
@@ -11367,38 +12290,38 @@
         </is>
       </c>
       <c r="N24" s="3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Παύλου Τίνα</t>
+          <t>Παλιος Νίκος</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΑΜΔΗ</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Λευκωσία</t>
+          <t>Πάφος</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Τίνα Παύλου - Tina Pavlou</t>
+          <t>Νίκος Παλιός</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>802383349636152</t>
+          <t>97122001685</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>35380689674908199</t>
+          <t>2081720626024053</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -11408,7 +12331,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -11416,54 +12339,46 @@
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>3,000–3,999</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>0–99</t>
-        </is>
-      </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
       <c r="N25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Στυλιανού Μάριος</t>
+          <t>Παλιος Νίκος</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΑΜΔΗ</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Λευκωσία</t>
+          <t>Πάφος</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Elpidios Christodoulou Officiaӏ</t>
+          <t>Νίκος Παλιός</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>842905035583022</t>
+          <t>97122001685</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>975708351876461</t>
+          <t>2387918571705884</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -11478,7 +12393,7 @@
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr"/>
@@ -11490,38 +12405,38 @@
         </is>
       </c>
       <c r="N26" s="3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Ελληνας Σάββας</t>
+          <t>Βραχιμη Έλενα</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ΑΜΔΗ</t>
+          <t>ΔΗΠΑ</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Πάφος</t>
+          <t>Λευκωσία</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Έλληνας Σάββας</t>
+          <t>elena.vrachimi</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>865790916625202</t>
+          <t>989853364206023</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>4446806865575192</t>
+          <t>1475766074023981</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -11531,7 +12446,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -11542,175 +12457,6 @@
         </is>
       </c>
       <c r="N27" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>Παλιος Νίκος</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>ΑΜΔΗ</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Πάφος</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>Νίκος Παλιός</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>97122001685</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>2081720626024053</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="J28" s="3" t="inlineStr"/>
-      <c r="K28" s="3" t="inlineStr"/>
-      <c r="L28" s="3" t="n"/>
-      <c r="M28" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N28" s="3" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Παλιος Νίκος</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>ΑΜΔΗ</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Πάφος</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Νίκος Παλιός</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>97122001685</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>2387918571705884</t>
-        </is>
-      </c>
-      <c r="G29" s="5" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N29" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>Βραχιμη Έλενα</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>ΔΗΠΑ</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Λευκωσία</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>elena.vrachimi</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>989853364206023</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>1475766074023981</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="I30" s="3" t="n"/>
-      <c r="J30" s="3" t="inlineStr"/>
-      <c r="K30" s="3" t="inlineStr"/>
-      <c r="L30" s="3" t="n"/>
-      <c r="M30" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="N30" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -11742,9 +12488,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto(CY): 3h refresh 2026-05-16T11:05Z
</commit_message>
<xml_diff>
--- a/daily_report_2026-05-16.xlsx
+++ b/daily_report_2026-05-16.xlsx
@@ -9951,8 +9951,6 @@
           <t>2026-05-05</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
       <c r="M71" t="inlineStr">
         <is>
           <t>2026-05-16 08:09</t>
@@ -10060,8 +10058,6 @@
           <t>2026-05-03</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
       <c r="M73" t="inlineStr">
         <is>
           <t>2026-05-16 08:05</t>
@@ -10169,8 +10165,6 @@
           <t>2026-05-05</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
       <c r="M75" t="inlineStr">
         <is>
           <t>2026-05-16 08:03</t>
@@ -10278,8 +10272,6 @@
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
       <c r="M77" t="inlineStr">
         <is>
           <t>2026-05-16 08:01</t>
@@ -10387,8 +10379,6 @@
           <t>2026-05-03</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
       <c r="M79" t="inlineStr">
         <is>
           <t>2026-05-16 08:01</t>
@@ -10496,8 +10486,6 @@
           <t>2026-05-11</t>
         </is>
       </c>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
       <c r="M81" t="inlineStr">
         <is>
           <t>2026-05-16 08:01</t>
@@ -10596,8 +10584,6 @@
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
       <c r="M83" t="inlineStr">
         <is>
           <t>2026-05-16 07:51</t>
@@ -10696,8 +10682,6 @@
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
       <c r="M85" t="inlineStr">
         <is>
           <t>2026-05-16 07:48</t>
@@ -10801,8 +10785,6 @@
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
       <c r="M87" t="inlineStr">
         <is>
           <t>2026-05-16 07:47</t>

</xml_diff>

<commit_message>
auto(CY): 3h refresh 2026-05-16T16:09Z
</commit_message>
<xml_diff>
--- a/daily_report_2026-05-16.xlsx
+++ b/daily_report_2026-05-16.xlsx
@@ -456,12 +456,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M92"/>
+  <dimension ref="A1:M104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
@@ -6130,6 +6130,752 @@
       <c r="M92" s="3" t="inlineStr">
         <is>
           <t>2026-05-16 05:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Τσαγγάρης Ανδρέας</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>ΣΗΚΟΥ ΠΑΝΩ</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Αντρέας Τσαγγάρης - ΣΗΚΟΥ ΠΑΝΩ</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>1116029114925274</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>965092452908208</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>5,000–5,999</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>Μενελαου Ελένη</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Αμμόχωστος</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>Eλένη Μενελάου/Eleni Menelaou</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>1317833338353731</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>955755290411400</t>
+        </is>
+      </c>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="J94" s="3" t="inlineStr">
+        <is>
+          <t>1,000–1,999</t>
+        </is>
+      </c>
+      <c r="K94" s="3" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="L94" s="3" t="n"/>
+      <c r="M94" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Παλιος Νίκος</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Νίκος Παλιός</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>97122001685</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>2387918571705884</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>Λαούρης Γιάννης</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>Yiannis Laouris</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>747263451806187</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>26858113073822656</t>
+        </is>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="I96" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="J96" s="3" t="inlineStr">
+        <is>
+          <t>10,000–14,999</t>
+        </is>
+      </c>
+      <c r="K96" s="3" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="L96" s="3" t="n"/>
+      <c r="M96" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Λαούρης Γιάννης</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Yiannis Laouris</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>747263451806187</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>3658020847678930</t>
+        </is>
+      </c>
+      <c r="G97" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>10,000–14,999</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>Κορύτσα Μαρία</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>ΕΛΑΜ</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>Αμμόχωστος</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>Μαρία Κορυτσά</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>636019372933735</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>813726091505369</t>
+        </is>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H98" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="I98" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="J98" s="3" t="inlineStr">
+        <is>
+          <t>1,000–1,999</t>
+        </is>
+      </c>
+      <c r="K98" s="3" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="L98" s="3" t="n"/>
+      <c r="M98" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Παύλου Τίνα</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Τίνα Παύλου - Tina Pavlou</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>802383349636152</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>35380689674908199</t>
+        </is>
+      </c>
+      <c r="G99" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>3,000–3,999</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>Αθανασιάδης Ζαχαρίας</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>ΕΛΑΜ</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>Ζαχαρίας Αθανασιάδης</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>146231858570802</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t>1330888802244834</t>
+        </is>
+      </c>
+      <c r="G100" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H100" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="I100" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J100" s="3" t="inlineStr">
+        <is>
+          <t>25,000–29,999</t>
+        </is>
+      </c>
+      <c r="K100" s="3" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="L100" s="3" t="n"/>
+      <c r="M100" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Χαμπούλλας Ευγένιος</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>ΕΛΑΜ</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>157660994287097</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>982291754490345</t>
+        </is>
+      </c>
+      <c r="G101" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>4,000–4,999</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>Χαμπούλλας Ευγένιος</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>ΕΛΑΜ</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>157660994287097</t>
+        </is>
+      </c>
+      <c r="F102" s="3" t="inlineStr">
+        <is>
+          <t>3040860612787824</t>
+        </is>
+      </c>
+      <c r="G102" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H102" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="I102" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J102" s="3" t="inlineStr">
+        <is>
+          <t>15,000–19,999</t>
+        </is>
+      </c>
+      <c r="K102" s="3" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="L102" s="3" t="n"/>
+      <c r="M102" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Χαμπούλλας Ευγένιος</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>ΕΛΑΜ</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>157660994287097</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>1533738934832768</t>
+        </is>
+      </c>
+      <c r="G103" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>3,000–3,999</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>Αποστόλου Ανδρέας</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΚΟ</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>Λάρνακα</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>Ανδρέας Αποστόλου</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>502944236549149</t>
+        </is>
+      </c>
+      <c r="F104" s="3" t="inlineStr">
+        <is>
+          <t>2026180128318814</t>
+        </is>
+      </c>
+      <c r="G104" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H104" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="I104" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="J104" s="3" t="inlineStr">
+        <is>
+          <t>8,000–8,999</t>
+        </is>
+      </c>
+      <c r="K104" s="3" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="L104" s="3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M104" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:45</t>
         </is>
       </c>
     </row>
@@ -6226,6 +6972,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G104" r:id="rId103"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6237,7 +6995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M87"/>
+  <dimension ref="A1:M98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -10788,6 +11546,557 @@
       <c r="M87" t="inlineStr">
         <is>
           <t>2026-05-16 07:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>Κυριακου Δημήτρης</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>ΑΛΜΑ</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>Parasita Enterprises</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>580616538466482</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>1436977004866337</t>
+        </is>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H88" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I88" s="3" t="n"/>
+      <c r="J88" s="3" t="inlineStr"/>
+      <c r="K88" s="3" t="inlineStr"/>
+      <c r="L88" s="3" t="n"/>
+      <c r="M88" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Άσπρης Άδαμος</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>ΔΗΚΟ</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Κερύνεια</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Adamos Aspris - Αδάμος Ασπρής</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>1544889622506869</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>1338561791485630</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr"/>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>Χατζηπαναγή Αρτέμης</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>ΕΝΕΡΓΟΙ ΠΟΛΙΤΕΣ</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>Αρτέμης Χατζηπαναγή</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>111255711940633</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>2207733500040396</t>
+        </is>
+      </c>
+      <c r="G90" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H90" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I90" s="3" t="n"/>
+      <c r="J90" s="3" t="inlineStr"/>
+      <c r="K90" s="3" t="inlineStr"/>
+      <c r="L90" s="3" t="n"/>
+      <c r="M90" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Παπαδοπουλος Γεώργιος</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>ΔΗΚΟ</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Λεμεσός</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Γεώργιος Παπαδόπουλος-Georgios Papadopoulos</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>101463311965634</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>27016679577962178</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>Παλιος Νίκος</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>Νίκος Παλιός</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>97122001685</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>1173276544896604</t>
+        </is>
+      </c>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H92" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I92" s="3" t="n"/>
+      <c r="J92" s="3" t="inlineStr"/>
+      <c r="K92" s="3" t="inlineStr"/>
+      <c r="L92" s="3" t="n"/>
+      <c r="M92" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Παλιος Νίκος</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Νίκος Παλιός</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>97122001685</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>1689103622409841</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>Παλιος Νίκος</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>Νίκος Παλιός</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>97122001685</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>2115554879176833</t>
+        </is>
+      </c>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I94" s="3" t="n"/>
+      <c r="J94" s="3" t="inlineStr"/>
+      <c r="K94" s="3" t="inlineStr"/>
+      <c r="L94" s="3" t="n"/>
+      <c r="M94" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Παλιος Νίκος</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Πάφος</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Νίκος Παλιός</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>97122001685</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>1251066740209941</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>Λαούρης Γιάννης</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>ΑΜΔΗ</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>Yiannis Laouris</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>747263451806187</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>978352818516825</t>
+        </is>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I96" s="3" t="n"/>
+      <c r="J96" s="3" t="inlineStr"/>
+      <c r="K96" s="3" t="inlineStr"/>
+      <c r="L96" s="3" t="n"/>
+      <c r="M96" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Παύλου Τίνα</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Τίνα Παύλου - Tina Pavlou</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>802383349636152</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>2229818011180300</t>
+        </is>
+      </c>
+      <c r="G97" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>Παύλου Τίνα</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΣΥ</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>Τίνα Παύλου - Tina Pavlou</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>802383349636152</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>1638625114089691</t>
+        </is>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H98" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I98" s="3" t="n"/>
+      <c r="J98" s="3" t="inlineStr"/>
+      <c r="K98" s="3" t="inlineStr"/>
+      <c r="L98" s="3" t="n"/>
+      <c r="M98" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 15:47</t>
         </is>
       </c>
     </row>
@@ -10879,6 +12188,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G98" r:id="rId97"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10890,19 +12210,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
@@ -10984,32 +12304,32 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Στυλιανού Μάριος</t>
+          <t>Βουτηρου Σάββας</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>ΑΛΜΑ</t>
+          <t>ΣΗΚΟΥ ΠΑΝΩ</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Λευκωσία</t>
+          <t>Αμμόχωστος</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Μάριος Στυλιανού</t>
+          <t>Σαββας Βουτήρου - Savvas Voutirou</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>1007793342425297</t>
+          <t>100936455330537</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>1696038684870609</t>
+          <t>1299002585765427</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -11019,14 +12339,10 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="n"/>
       <c r="J2" s="3" t="inlineStr"/>
       <c r="K2" s="3" t="inlineStr"/>
       <c r="L2" s="3" t="n"/>
@@ -11036,38 +12352,38 @@
         </is>
       </c>
       <c r="N2" s="3" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Στυλιανού Μάριος</t>
+          <t>Παπαδοπουλος Γεώργιος</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ΑΛΜΑ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Λευκωσία</t>
+          <t>Λεμεσός</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Μάριος Στυλιανού</t>
+          <t>Γεώργιος Παπαδόπουλος-Georgios Papadopoulos</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1007793342425297</t>
+          <t>101463311965634</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>923719130700237</t>
+          <t>27016679577962178</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
@@ -11077,12 +12393,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -11093,38 +12404,38 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Βουτηρου Σάββας</t>
+          <t>Γεωργιάδης Δήμος</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>ΣΗΚΟΥ ΠΑΝΩ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Αμμόχωστος</t>
+          <t>Κερύνεια</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Σαββας Βουτήρου - Savvas Voutirou</t>
+          <t>Δήμος Γεωργιάδης</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>100936455330537</t>
+          <t>107513542170251</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>1299002585765427</t>
+          <t>1286848666896373</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -11134,7 +12445,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="I4" s="3" t="n"/>
@@ -11147,18 +12458,18 @@
         </is>
       </c>
       <c r="N4" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Γεωργιάδης Δήμος</t>
+          <t>Άσπρης Άδαμος</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -11168,17 +12479,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Δήμος Γεωργιάδης</t>
+          <t>Adamos Aspris - Αδάμος Ασπρής</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>107513542170251</t>
+          <t>1544889622506869</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1286848666896373</t>
+          <t>1287137836934355</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -11188,7 +12499,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -11199,18 +12510,18 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Γεωργιάδης Δήμος</t>
+          <t>Άσπρης Άδαμος</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -11220,17 +12531,17 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Δήμος Γεωργιάδης</t>
+          <t>Adamos Aspris - Αδάμος Ασπρής</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>107513542170251</t>
+          <t>1544889622506869</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>1303700075068172</t>
+          <t>1338561791485630</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -11240,14 +12551,10 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="inlineStr"/>
       <c r="K6" s="3" t="inlineStr"/>
       <c r="L6" s="3" t="n"/>
@@ -11257,13 +12564,13 @@
         </is>
       </c>
       <c r="N6" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Αθανασιάδης Ζαχαρίας</t>
+          <t>Χαμπούλλας Ευγένιος</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -11278,17 +12585,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Ζαχαρίας Αθανασιάδης</t>
+          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>146231858570802</t>
+          <t>157660994287097</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1330888802244834</t>
+          <t>1032725159187111</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -11298,62 +12605,49 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
           <t>2026-05-15</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>25,000–29,999</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>0–99</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t>2026-05-14</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Άσπρης Άδαμος</t>
+          <t>Χαμπούλλας Ευγένιος</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΕΛΑΜ</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Κερύνεια</t>
+          <t>Λεμεσός</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Adamos Aspris - Αδάμος Ασπρής</t>
+          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>1544889622506869</t>
+          <t>157660994287097</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>1287137836934355</t>
+          <t>3440749736091343</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -11363,7 +12657,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="I8" s="3" t="n"/>
@@ -11376,38 +12670,38 @@
         </is>
       </c>
       <c r="N8" s="3" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Χαμπούλλας Ευγένιος</t>
+          <t>Αποστόλου Ανδρέας</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ΕΛΑΜ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Λεμεσός</t>
+          <t>Λάρνακα</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
+          <t>Ανδρέας Αποστόλου</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>157660994287097</t>
+          <t>502944236549149</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1032725159187111</t>
+          <t>1695784821453815</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -11428,38 +12722,38 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Χαμπούλλας Ευγένιος</t>
+          <t>Σαββίδης Χρύσανθος</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>ΕΛΑΜ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Λεμεσός</t>
+          <t>Πάφος</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
+          <t>Χρύσανθος Σαββίδης</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>157660994287097</t>
+          <t>556192687867978</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>3440749736091343</t>
+          <t>2071083287123146</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -11469,7 +12763,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="I10" s="3" t="n"/>
@@ -11482,38 +12776,38 @@
         </is>
       </c>
       <c r="N10" s="3" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Αποστόλου Ανδρέας</t>
+          <t>Φελλάς Μιχάλης</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Λάρνακα</t>
+          <t>Λεμεσός</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Ανδρέας Αποστόλου</t>
+          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>502944236549149</t>
+          <t>574683626048556</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1695784821453815</t>
+          <t>2460936817680213</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -11528,7 +12822,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -11539,38 +12833,38 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>21</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Σαββίδης Χρύσανθος</t>
+          <t>Ευαγγελου Αργυρός</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Πάφος</t>
+          <t>Λάρνακα</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Χρύσανθος Σαββίδης</t>
+          <t>Αργυρός Ευαγγέλου - Argyros Evangelou</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>556192687867978</t>
+          <t>595915680800838</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>2071083287123146</t>
+          <t>2039508410305874</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -11580,7 +12874,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="I12" s="3" t="n"/>
@@ -11593,38 +12887,38 @@
         </is>
       </c>
       <c r="N12" s="3" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης</t>
+          <t>Κορύτσα Μαρία</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΕΛΑΜ</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Λεμεσός</t>
+          <t>Αμμόχωστος</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+          <t>Μαρία Κορυτσά</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>574683626048556</t>
+          <t>636019372933735</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2460936817680213</t>
+          <t>1296943101983207</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -11639,7 +12933,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -11650,38 +12944,38 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Ευαγγελου Αργυρός</t>
+          <t>Λαούρης Γιάννης</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΑΜΔΗ</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Λάρνακα</t>
+          <t>Λευκωσία</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Αργυρός Ευαγγέλου - Argyros Evangelou</t>
+          <t>Yiannis Laouris</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>595915680800838</t>
+          <t>747263451806187</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>2039508410305874</t>
+          <t>978352818516825</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -11691,7 +12985,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="I14" s="3" t="n"/>
@@ -11704,38 +12998,38 @@
         </is>
       </c>
       <c r="N14" s="3" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Κορύτσα Μαρία</t>
+          <t>Φελλάς Μιχάλης</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ΕΛΑΜ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Αμμόχωστος</t>
+          <t>Λεμεσός</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Μαρία Κορυτσά</t>
+          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>636019372933735</t>
+          <t>754699914874253</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1296943101983207</t>
+          <t>1271006601866511</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -11746,6 +13040,11 @@
       <c r="H15" t="inlineStr">
         <is>
           <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -11756,38 +13055,38 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>15</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Κορύτσα Μαρία</t>
+          <t>Φελλάς Μιχάλης</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>ΕΛΑΜ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Αμμόχωστος</t>
+          <t>Λεμεσός</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Μαρία Κορυτσά</t>
+          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>636019372933735</t>
+          <t>754699914874253</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>813726091505369</t>
+          <t>2150144575829086</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -11797,24 +13096,16 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>1,000–1,999</t>
-        </is>
-      </c>
-      <c r="K16" s="3" t="inlineStr">
-        <is>
-          <t>0–99</t>
-        </is>
-      </c>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr"/>
+      <c r="K16" s="3" t="inlineStr"/>
       <c r="L16" s="3" t="n"/>
       <c r="M16" s="3" t="inlineStr">
         <is>
@@ -11822,13 +13113,13 @@
         </is>
       </c>
       <c r="N16" s="3" t="n">
-        <v>15</v>
+        <v>79</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης</t>
+          <t>Παύλου Τίνα</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -11838,22 +13129,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Λεμεσός</t>
+          <t>Λευκωσία</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+          <t>Τίνα Παύλου - Tina Pavlou</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>754699914874253</t>
+          <t>802383349636152</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1271006601866511</t>
+          <t>2718683645168629</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -11863,12 +13154,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -11879,13 +13165,13 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης</t>
+          <t>Παύλου Τίνα</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -11895,22 +13181,22 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Λεμεσός</t>
+          <t>Λευκωσία</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+          <t>Τίνα Παύλου - Tina Pavlou</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>754699914874253</t>
+          <t>802383349636152</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>2150144575829086</t>
+          <t>2229818011180300</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -11920,14 +13206,10 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="n"/>
       <c r="J18" s="3" t="inlineStr"/>
       <c r="K18" s="3" t="inlineStr"/>
       <c r="L18" s="3" t="n"/>
@@ -11937,7 +13219,7 @@
         </is>
       </c>
       <c r="N18" s="3" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19">
@@ -11968,7 +13250,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2718683645168629</t>
+          <t>1638625114089691</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
@@ -11989,7 +13271,7 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20">
@@ -12047,7 +13329,7 @@
         </is>
       </c>
       <c r="N20" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
@@ -12099,7 +13381,7 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22">
@@ -12153,38 +13435,38 @@
         </is>
       </c>
       <c r="N22" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Παύλου Τίνα</t>
+          <t>Παλιος Νίκος</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΑΜΔΗ</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Λευκωσία</t>
+          <t>Πάφος</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Τίνα Παύλου - Tina Pavlou</t>
+          <t>Νίκος Παλιός</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>802383349636152</t>
+          <t>97122001685</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>35380689674908199</t>
+          <t>1173276544896604</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -12194,24 +13476,11 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>3,000–3,999</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>0–99</t>
-        </is>
-      </c>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="M23" t="inlineStr">
         <is>
           <t>2026-05-14</t>
@@ -12224,7 +13493,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Ελληνας Σάββας</t>
+          <t>Παλιος Νίκος</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -12239,17 +13508,17 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Έλληνας Σάββας</t>
+          <t>Νίκος Παλιός</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>865790916625202</t>
+          <t>97122001685</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>4446806865575192</t>
+          <t>1689103622409841</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -12259,7 +13528,7 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="I24" s="3" t="n"/>
@@ -12272,7 +13541,7 @@
         </is>
       </c>
       <c r="N24" s="3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25">
@@ -12303,7 +13572,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2081720626024053</t>
+          <t>2115554879176833</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -12313,12 +13582,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -12329,7 +13593,7 @@
         </is>
       </c>
       <c r="N25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26">
@@ -12360,7 +13624,7 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>2387918571705884</t>
+          <t>1251066740209941</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -12370,14 +13634,10 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
           <t>2026-05-16</t>
         </is>
       </c>
+      <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="inlineStr"/>
       <c r="K26" s="3" t="inlineStr"/>
       <c r="L26" s="3" t="n"/>
@@ -12387,38 +13647,38 @@
         </is>
       </c>
       <c r="N26" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Βραχιμη Έλενα</t>
+          <t>Παλιος Νίκος</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ΔΗΠΑ</t>
+          <t>ΑΜΔΗ</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Λευκωσία</t>
+          <t>Πάφος</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>elena.vrachimi</t>
+          <t>Νίκος Παλιός</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>989853364206023</t>
+          <t>97122001685</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>1475766074023981</t>
+          <t>2081720626024053</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -12428,7 +13688,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -12439,6 +13704,60 @@
         </is>
       </c>
       <c r="N27" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Βραχιμη Έλενα</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>ΔΗΠΑ</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Λευκωσία</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>elena.vrachimi</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>989853364206023</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>1475766074023981</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="inlineStr"/>
+      <c r="K28" s="3" t="inlineStr"/>
+      <c r="L28" s="3" t="n"/>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="N28" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -12470,6 +13789,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>